<commit_message>
Show complete unqualified initial P21 counts in metric 4
</commit_message>
<xml_diff>
--- a/pre_experiment/results/2026-10-21/metrics.xlsx
+++ b/pre_experiment/results/2026-10-21/metrics.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot comparison" sheetId="1" r:id="R43b8f01fa08b4c88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot comparison" sheetId="1" r:id="R7c2bb12651e44019"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -485,23 +485,23 @@
         <x:v>Initial: pairs 26, instances 4802, distinct rules 10; Final: pairs 24, instances 3940, distinct rules 9</x:v>
       </x:c>
       <x:c r="D10" s="11" t="str">
-        <x:v>Initial: pairs Unavailable, instances Unavailable, distinct rules Unavailable; Final: pairs 26, instances 4708, distinct rules 10
-Unqualified observed initial: 39 pairs, 458163 instances (not scored)</x:v>
+        <x:v>Unqualified observed initial: 39 pairs, 458,163 instances, 12 distinct rules (not scored)
+Initial: pairs Unavailable, instances Unavailable, distinct rules Unavailable; Final: pairs 26, instances 4708, distinct rules 10</x:v>
       </x:c>
       <x:c r="E10" s="11" t="str">
         <x:v>Initial: pairs 26, instances 4822, distinct rules 10; Final: pairs 24, instances 4074, distinct rules 9</x:v>
       </x:c>
       <x:c r="F10" s="11" t="str">
-        <x:v>Initial: pairs Unavailable, instances Unavailable, distinct rules Unavailable; Final: pairs 26, instances 4822, distinct rules 10
-Unqualified observed initial: 26 pairs, 4822 instances (not scored)</x:v>
+        <x:v>Unqualified observed initial: 26 pairs, 4,822 instances, 10 distinct rules (not scored)
+Initial: pairs Unavailable, instances Unavailable, distinct rules Unavailable; Final: pairs 26, instances 4822, distinct rules 10</x:v>
       </x:c>
       <x:c r="G10" s="11" t="str">
         <x:v>Initial: pairs 49, instances 1541131, distinct rules 7; Final: pairs 15, instances 35, distinct rules 4</x:v>
       </x:c>
       <x:c r="H10" s="11" t="str">
-        <x:v>Initial: pairs Unavailable, instances Unavailable, distinct rules Unavailable; Final: pairs Unavailable, instances Unavailable, distinct rules Unavailable
-Unqualified observed initial: 77 pairs, 945842 instances (not scored)
-Unqualified observed final: 63 pairs, 694458 instances (not scored)</x:v>
+        <x:v>Unqualified observed initial: 77 pairs, 945,842 instances, 10 distinct rules (not scored)
+Unqualified observed final: 63 pairs, 694,458 instances, 9 distinct rules (not scored)
+Initial: pairs Unavailable, instances Unavailable, distinct rules Unavailable; Final: pairs Unavailable, instances Unavailable, distinct rules Unavailable</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="80" customHeight="1">

</xml_diff>